<commit_message>
added new data for 2026 in opm and dcr
</commit_message>
<xml_diff>
--- a/data/Departamento_de_correccion_y_rehabilitacion/dcr_Alternos.xlsx
+++ b/data/Departamento_de_correccion_y_rehabilitacion/dcr_Alternos.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Departamento_de_correccion_y_rehabilitacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DE7452-985F-4EBF-88D9-63C731DC4619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="8688" yWindow="2088" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -381,15 +382,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -403,7 +404,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -417,7 +418,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -431,7 +432,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2025</v>
       </c>
@@ -445,7 +446,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2025</v>
       </c>
@@ -459,7 +460,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -470,10 +471,10 @@
         <v>5</v>
       </c>
       <c r="D6">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -484,10 +485,10 @@
         <v>5</v>
       </c>
       <c r="D7">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -501,7 +502,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -515,7 +516,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2025</v>
       </c>
@@ -529,7 +530,7 @@
         <v>1248</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2025</v>
       </c>
@@ -543,7 +544,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -554,10 +555,10 @@
         <v>6</v>
       </c>
       <c r="D12">
-        <v>1330</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -568,7 +569,7 @@
         <v>6</v>
       </c>
       <c r="D13">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>